<commit_message>
docs: update test cases mapping after login parameterization
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1. Click Close Welcome Banner on the Welcome banner. 2. Click Me want it! on the cookie banner.</t>
+          <t>1. Click Close Welcome Banner on the Welcome banner. 2. Click Me want it! (Dismiss cookie message) on the cookie banner.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>User is redirected to the main page. Account menu shows the user email.</t>
+          <t>User is redirected to the search page with the product list. Account menu shows the user email.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>tests/login.spec.js › should log in with valid credentials</t>
+          <t>tests/login.spec.js › should handle login: valid credentials</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>tests/login.spec.js › should reject login: wrong password</t>
+          <t>tests/login.spec.js › should handle login: wrong password</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Login page is open</t>
+          <t>Registered test user exists. Banners are dismissed. Login form is open.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>tests/login.spec.js › should reject login: non-existing email</t>
+          <t>tests/login.spec.js › should handle login: non-existing email</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Login page is open</t>
+          <t>Banners are dismissed. Login form is open.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>tests/login.spec.js › should block login with empty email</t>
+          <t>tests/login.spec.js › should handle login: empty email</t>
         </is>
       </c>
     </row>
@@ -774,7 +774,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Login page is open</t>
+          <t>Registered test user exists. Banners are dismissed. Login form is open.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Login page is open</t>
+          <t>Banners are dismissed. Login form is open.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Main page is open</t>
+          <t>Banners are dismissed. Main page is open.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Main page is open</t>
+          <t>Banners are dismissed. Main page is open.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">

</xml_diff>